<commit_message>
Added new RDF data schemes and visual schemes for employment-table24-25, fixed XLSX spreadsheets for employment-table24-25
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table24.xlsx
+++ b/sources/table_normalization/xlsx/employment-table24.xlsx
@@ -192,16 +192,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -525,7 +529,7 @@
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -533,29 +537,29 @@
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="5">
         <v>2023</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="5" t="s">
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="6" t="s">
         <v>5</v>
       </c>
       <c r="H5" s="4" t="s">
@@ -565,42 +569,42 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="5" t="s">
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="6" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="4"/>
+      <c r="G7" s="7"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1388,7 +1392,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="8" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1741,7 +1745,7 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="8" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>